<commit_message>
Adding checking the file exists or not
</commit_message>
<xml_diff>
--- a/dist/report_June.xlsx
+++ b/dist/report_June.xlsx
@@ -19,7 +19,7 @@
     <t>Accommodation Report</t>
   </si>
   <si>
-    <t>June</t>
+    <t>june</t>
   </si>
   <si>
     <t>Gender</t>
@@ -325,11 +325,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="306308224"/>
-        <c:axId val="306309760"/>
+        <c:axId val="299492480"/>
+        <c:axId val="299494016"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="306308224"/>
+        <c:axId val="299492480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -338,7 +338,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="306309760"/>
+        <c:crossAx val="299494016"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -346,7 +346,7 @@
         <c:noMultiLvlLbl val="1"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="306309760"/>
+        <c:axId val="299494016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -357,7 +357,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="306308224"/>
+        <c:crossAx val="299492480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>